<commit_message>
Updated data for care (v69)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_care.xlsx
+++ b/src/data/routekaart_status_care.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63522D24-3023-49AC-8CC0-DDC47F5E0429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D24ECE-5FB4-4665-81F9-F8E1859F465C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5265" yWindow="4110" windowWidth="38700" windowHeight="15285" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="3195" yWindow="1590" windowWidth="23535" windowHeight="19020" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="616" uniqueCount="311">
   <si>
     <t>Status inleveren routekaart</t>
   </si>
@@ -943,13 +943,25 @@
     <t>Stichting ZZG zorggroep</t>
   </si>
   <si>
-    <t>Stichting Kind &amp; Co Ludens</t>
-  </si>
-  <si>
     <t>Van Neynselstichting</t>
   </si>
   <si>
     <t xml:space="preserve">Vereen </t>
+  </si>
+  <si>
+    <t>Stichting Christelijke Zorgorganisatie Norschoten</t>
+  </si>
+  <si>
+    <t>Stichting De Tussenvoorziening</t>
+  </si>
+  <si>
+    <t>Stichting Zorggroep De Betuwe</t>
+  </si>
+  <si>
+    <t>Stichting Zorgpartners Friesland (voorheen handelsnaam Noorderbreedte)</t>
+  </si>
+  <si>
+    <t>Stichting Buurtzorg Nederland</t>
   </si>
 </sst>
 </file>
@@ -1317,7 +1329,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F40E7E-2647-4F3F-8219-3AF753B4033B}">
-  <dimension ref="A1:B304"/>
+  <dimension ref="A1:B308"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="73.140625" customWidth="1"/>
@@ -1345,7 +1357,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1537,7 +1549,7 @@
         <v>38</v>
       </c>
       <c r="B27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -1681,7 +1693,7 @@
         <v>54</v>
       </c>
       <c r="B45" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -1873,7 +1885,7 @@
         <v>77</v>
       </c>
       <c r="B69" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -1966,31 +1978,31 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>89</v>
+        <v>306</v>
       </c>
       <c r="B81" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B82" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B83" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B84" t="s">
         <v>15</v>
@@ -1998,7 +2010,7 @@
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B85" t="s">
         <v>15</v>
@@ -2006,7 +2018,7 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B86" t="s">
         <v>15</v>
@@ -2014,7 +2026,7 @@
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B87" t="s">
         <v>15</v>
@@ -2022,15 +2034,15 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B88" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B89" t="s">
         <v>16</v>
@@ -2038,31 +2050,31 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B90" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B91" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B92" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B93" t="s">
         <v>15</v>
@@ -2070,7 +2082,7 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B94" t="s">
         <v>15</v>
@@ -2078,7 +2090,7 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>103</v>
+        <v>307</v>
       </c>
       <c r="B95" t="s">
         <v>15</v>
@@ -2086,7 +2098,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B96" t="s">
         <v>15</v>
@@ -2094,7 +2106,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B97" t="s">
         <v>15</v>
@@ -2102,7 +2114,7 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B98" t="s">
         <v>15</v>
@@ -2110,15 +2122,15 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B99" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B100" t="s">
         <v>15</v>
@@ -2126,7 +2138,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B101" t="s">
         <v>16</v>
@@ -2134,7 +2146,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B102" t="s">
         <v>15</v>
@@ -2142,7 +2154,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B103" t="s">
         <v>16</v>
@@ -2150,7 +2162,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B104" t="s">
         <v>15</v>
@@ -2158,7 +2170,7 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B105" t="s">
         <v>16</v>
@@ -2166,47 +2178,47 @@
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B106" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B107" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B108" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B109" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B110" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B111" t="s">
         <v>16</v>
@@ -2214,23 +2226,23 @@
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B112" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B113" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B114" t="s">
         <v>16</v>
@@ -2238,7 +2250,7 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B115" t="s">
         <v>15</v>
@@ -2246,15 +2258,15 @@
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B116" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B117" t="s">
         <v>15</v>
@@ -2262,7 +2274,7 @@
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B118" t="s">
         <v>15</v>
@@ -2270,7 +2282,7 @@
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B119" t="s">
         <v>15</v>
@@ -2278,7 +2290,7 @@
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B120" t="s">
         <v>15</v>
@@ -2286,7 +2298,7 @@
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B121" t="s">
         <v>15</v>
@@ -2294,7 +2306,7 @@
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B122" t="s">
         <v>15</v>
@@ -2302,7 +2314,7 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B123" t="s">
         <v>15</v>
@@ -2310,47 +2322,47 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B124" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B125" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B126" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B127" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B128" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B129" t="s">
         <v>15</v>
@@ -2358,15 +2370,15 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B130" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B131" t="s">
         <v>15</v>
@@ -2374,7 +2386,7 @@
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B132" t="s">
         <v>15</v>
@@ -2382,15 +2394,15 @@
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B133" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B134" t="s">
         <v>15</v>
@@ -2398,7 +2410,7 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B135" t="s">
         <v>16</v>
@@ -2406,15 +2418,15 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B136" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B137" t="s">
         <v>16</v>
@@ -2422,7 +2434,7 @@
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B138" t="s">
         <v>16</v>
@@ -2430,23 +2442,23 @@
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B139" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B140" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B141" t="s">
         <v>15</v>
@@ -2454,7 +2466,7 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B142" t="s">
         <v>15</v>
@@ -2462,15 +2474,15 @@
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B143" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B144" t="s">
         <v>15</v>
@@ -2478,15 +2490,15 @@
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B145" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B146" t="s">
         <v>15</v>
@@ -2494,7 +2506,7 @@
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B147" t="s">
         <v>15</v>
@@ -2502,15 +2514,15 @@
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B148" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B149" t="s">
         <v>15</v>
@@ -2518,23 +2530,23 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B150" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B151" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B152" t="s">
         <v>15</v>
@@ -2542,7 +2554,7 @@
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B153" t="s">
         <v>16</v>
@@ -2550,7 +2562,7 @@
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B154" t="s">
         <v>15</v>
@@ -2558,15 +2570,15 @@
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B155" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B156" t="s">
         <v>15</v>
@@ -2574,7 +2586,7 @@
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B157" t="s">
         <v>15</v>
@@ -2582,7 +2594,7 @@
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B158" t="s">
         <v>15</v>
@@ -2590,7 +2602,7 @@
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B159" t="s">
         <v>15</v>
@@ -2598,15 +2610,15 @@
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B160" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B161" t="s">
         <v>15</v>
@@ -2614,7 +2626,7 @@
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B162" t="s">
         <v>16</v>
@@ -2622,7 +2634,7 @@
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B163" t="s">
         <v>15</v>
@@ -2630,15 +2642,15 @@
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B164" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B165" t="s">
         <v>15</v>
@@ -2646,7 +2658,7 @@
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B166" t="s">
         <v>15</v>
@@ -2654,15 +2666,15 @@
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B167" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B168" t="s">
         <v>15</v>
@@ -2670,7 +2682,7 @@
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B169" t="s">
         <v>16</v>
@@ -2678,7 +2690,7 @@
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B170" t="s">
         <v>15</v>
@@ -2686,7 +2698,7 @@
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B171" t="s">
         <v>16</v>
@@ -2694,15 +2706,15 @@
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B172" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B173" t="s">
         <v>16</v>
@@ -2710,7 +2722,7 @@
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B174" t="s">
         <v>15</v>
@@ -2718,47 +2730,47 @@
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B175" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B176" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B177" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B178" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B179" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B180" t="s">
         <v>15</v>
@@ -2766,7 +2778,7 @@
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B181" t="s">
         <v>15</v>
@@ -2774,7 +2786,7 @@
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B182" t="s">
         <v>15</v>
@@ -2782,31 +2794,31 @@
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B183" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B184" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B185" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B186" t="s">
         <v>16</v>
@@ -2814,7 +2826,7 @@
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B187" t="s">
         <v>15</v>
@@ -2822,15 +2834,15 @@
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B188" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B189" t="s">
         <v>15</v>
@@ -2838,15 +2850,15 @@
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B190" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B191" t="s">
         <v>15</v>
@@ -2854,7 +2866,7 @@
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B192" t="s">
         <v>15</v>
@@ -2862,7 +2874,7 @@
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B193" t="s">
         <v>15</v>
@@ -2870,7 +2882,7 @@
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B194" t="s">
         <v>15</v>
@@ -2878,7 +2890,7 @@
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B195" t="s">
         <v>15</v>
@@ -2886,7 +2898,7 @@
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B196" t="s">
         <v>15</v>
@@ -2894,7 +2906,7 @@
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B197" t="s">
         <v>15</v>
@@ -2902,47 +2914,47 @@
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B198" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B199" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B200" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B201" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B202" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B203" t="s">
         <v>15</v>
@@ -2950,15 +2962,15 @@
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B204" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B205" t="s">
         <v>15</v>
@@ -2966,7 +2978,7 @@
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B206" t="s">
         <v>16</v>
@@ -2974,7 +2986,7 @@
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B207" t="s">
         <v>15</v>
@@ -2982,7 +2994,7 @@
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B208" t="s">
         <v>16</v>
@@ -2990,31 +3002,31 @@
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B209" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B210" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B211" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B212" t="s">
         <v>15</v>
@@ -3022,15 +3034,15 @@
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B213" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B214" t="s">
         <v>15</v>
@@ -3038,23 +3050,23 @@
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B215" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B216" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B217" t="s">
         <v>15</v>
@@ -3062,55 +3074,55 @@
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B218" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B219" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B220" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B221" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B222" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="223" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B223" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B224" t="s">
         <v>15</v>
@@ -3118,23 +3130,23 @@
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B225" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B226" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B227" t="s">
         <v>15</v>
@@ -3142,7 +3154,7 @@
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B228" t="s">
         <v>16</v>
@@ -3150,23 +3162,23 @@
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B229" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B230" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B231" t="s">
         <v>16</v>
@@ -3174,7 +3186,7 @@
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B232" t="s">
         <v>15</v>
@@ -3182,15 +3194,15 @@
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>21</v>
+        <v>239</v>
       </c>
       <c r="B233" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B234" t="s">
         <v>15</v>
@@ -3198,7 +3210,7 @@
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>242</v>
+        <v>21</v>
       </c>
       <c r="B235" t="s">
         <v>15</v>
@@ -3206,39 +3218,39 @@
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B236" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B237" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B238" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B239" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B240" t="s">
         <v>15</v>
@@ -3246,31 +3258,31 @@
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B241" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B242" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B243" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B244" t="s">
         <v>16</v>
@@ -3278,31 +3290,31 @@
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B245" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B246" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B247" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B248" t="s">
         <v>15</v>
@@ -3310,7 +3322,7 @@
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B249" t="s">
         <v>15</v>
@@ -3318,15 +3330,15 @@
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B250" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B251" t="s">
         <v>15</v>
@@ -3334,15 +3346,15 @@
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B252" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B253" t="s">
         <v>15</v>
@@ -3350,15 +3362,15 @@
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B254" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B255" t="s">
         <v>15</v>
@@ -3366,7 +3378,7 @@
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B256" t="s">
         <v>15</v>
@@ -3374,7 +3386,7 @@
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B257" t="s">
         <v>15</v>
@@ -3382,15 +3394,15 @@
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B258" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B259" t="s">
         <v>15</v>
@@ -3398,15 +3410,15 @@
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B260" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B261" t="s">
         <v>15</v>
@@ -3414,7 +3426,7 @@
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B262" t="s">
         <v>15</v>
@@ -3422,7 +3434,7 @@
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B263" t="s">
         <v>15</v>
@@ -3430,7 +3442,7 @@
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B264" t="s">
         <v>15</v>
@@ -3438,31 +3450,31 @@
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B265" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B266" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B267" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B268" t="s">
         <v>16</v>
@@ -3470,7 +3482,7 @@
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B269" t="s">
         <v>15</v>
@@ -3478,23 +3490,23 @@
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B270" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B271" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B272" t="s">
         <v>15</v>
@@ -3502,7 +3514,7 @@
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B273" t="s">
         <v>16</v>
@@ -3510,31 +3522,31 @@
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B274" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B275" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B276" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B277" t="s">
         <v>15</v>
@@ -3542,7 +3554,7 @@
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>285</v>
+        <v>308</v>
       </c>
       <c r="B278" t="s">
         <v>16</v>
@@ -3550,7 +3562,7 @@
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B279" t="s">
         <v>15</v>
@@ -3558,31 +3570,31 @@
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B280" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B281" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B282" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B283" t="s">
         <v>16</v>
@@ -3590,31 +3602,31 @@
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B284" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B285" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B286" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B287" t="s">
         <v>16</v>
@@ -3622,7 +3634,7 @@
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="B288" t="s">
         <v>15</v>
@@ -3630,23 +3642,23 @@
     </row>
     <row r="289" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B289" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="290" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B290" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="291" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B291" t="s">
         <v>15</v>
@@ -3654,15 +3666,15 @@
     </row>
     <row r="292" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="B292" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="293" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B293" t="s">
         <v>15</v>
@@ -3670,15 +3682,15 @@
     </row>
     <row r="294" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B294" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="295" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B295" t="s">
         <v>15</v>
@@ -3686,15 +3698,15 @@
     </row>
     <row r="296" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="B296" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="297" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="B297" t="s">
         <v>15</v>
@@ -3702,15 +3714,15 @@
     </row>
     <row r="298" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>10</v>
+        <v>301</v>
       </c>
       <c r="B298" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="299" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B299" t="s">
         <v>15</v>
@@ -3718,7 +3730,7 @@
     </row>
     <row r="300" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B300" t="s">
         <v>15</v>
@@ -3726,33 +3738,65 @@
     </row>
     <row r="301" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>4</v>
+        <v>310</v>
       </c>
       <c r="B301" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="302" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B302" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>8</v>
+        <v>304</v>
       </c>
       <c r="B303" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="304" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
+        <v>305</v>
+      </c>
+      <c r="B304" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
+        <v>4</v>
+      </c>
+      <c r="B305" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
+        <v>5</v>
+      </c>
+      <c r="B306" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
+        <v>8</v>
+      </c>
+      <c r="B307" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
         <v>27</v>
       </c>
-      <c r="B304" t="s">
+      <c r="B308" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated data for care (v71)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_care.xlsx
+++ b/src/data/routekaart_status_care.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E38D95F-F817-4548-99A0-A4F012E092AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357B885A-BF94-45AB-9A3C-602A95A47A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="4770" windowWidth="32840" windowHeight="14400" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="17250" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="317">
   <si>
     <t>Status inleveren routekaart</t>
   </si>
@@ -968,6 +968,18 @@
   </si>
   <si>
     <t>Stichting Zorgorganisatie NiKo</t>
+  </si>
+  <si>
+    <t>Stichting Reinaerde</t>
+  </si>
+  <si>
+    <t>Stichting zorggroep Maas &amp; Waal</t>
+  </si>
+  <si>
+    <t>Stichting Zorggroep Noordwest-Veluwe Holding</t>
+  </si>
+  <si>
+    <t>VraagPlus B.V.</t>
   </si>
 </sst>
 </file>
@@ -1335,14 +1347,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F40E7E-2647-4F3F-8219-3AF753B4033B}">
-  <dimension ref="A1:B310"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B314"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="73.1796875" customWidth="1"/>
-    <col min="2" max="2" width="31.453125" customWidth="1"/>
+    <col min="1" max="1" width="73.140625" customWidth="1"/>
+    <col min="2" max="2" width="31.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1350,7 +1362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1358,7 +1370,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1366,7 +1378,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -1374,7 +1386,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1382,7 +1394,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -1390,7 +1402,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1398,7 +1410,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -1406,7 +1418,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1414,7 +1426,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -1422,7 +1434,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -1430,7 +1442,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1438,7 +1450,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1446,7 +1458,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1454,7 +1466,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1462,7 +1474,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -1470,7 +1482,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1478,7 +1490,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1486,7 +1498,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1494,7 +1506,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -1502,7 +1514,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -1510,7 +1522,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -1518,7 +1530,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -1526,7 +1538,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>36</v>
       </c>
@@ -1534,7 +1546,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>6</v>
       </c>
@@ -1542,7 +1554,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>310</v>
       </c>
@@ -1550,7 +1562,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1558,7 +1570,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -1566,7 +1578,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>39</v>
       </c>
@@ -1574,7 +1586,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -1582,7 +1594,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>41</v>
       </c>
@@ -1590,7 +1602,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -1598,7 +1610,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -1606,7 +1618,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>44</v>
       </c>
@@ -1614,7 +1626,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -1622,7 +1634,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>46</v>
       </c>
@@ -1630,7 +1642,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -1638,7 +1650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -1646,7 +1658,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>7</v>
       </c>
@@ -1654,7 +1666,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>49</v>
       </c>
@@ -1662,7 +1674,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -1670,7 +1682,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>50</v>
       </c>
@@ -1678,7 +1690,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>51</v>
       </c>
@@ -1686,7 +1698,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -1694,7 +1706,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -1702,7 +1714,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -1710,7 +1722,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -1718,7 +1730,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>56</v>
       </c>
@@ -1726,7 +1738,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>25</v>
       </c>
@@ -1734,7 +1746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>57</v>
       </c>
@@ -1742,7 +1754,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>58</v>
       </c>
@@ -1750,7 +1762,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>59</v>
       </c>
@@ -1758,7 +1770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>60</v>
       </c>
@@ -1766,7 +1778,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -1774,7 +1786,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>62</v>
       </c>
@@ -1782,7 +1794,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>63</v>
       </c>
@@ -1790,7 +1802,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>64</v>
       </c>
@@ -1798,7 +1810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>65</v>
       </c>
@@ -1806,7 +1818,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>66</v>
       </c>
@@ -1814,7 +1826,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>67</v>
       </c>
@@ -1822,7 +1834,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>68</v>
       </c>
@@ -1830,7 +1842,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>69</v>
       </c>
@@ -1838,7 +1850,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>70</v>
       </c>
@@ -1846,7 +1858,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>71</v>
       </c>
@@ -1854,7 +1866,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>72</v>
       </c>
@@ -1862,7 +1874,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>73</v>
       </c>
@@ -1870,7 +1882,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>74</v>
       </c>
@@ -1878,7 +1890,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>75</v>
       </c>
@@ -1886,7 +1898,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>76</v>
       </c>
@@ -1894,7 +1906,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>77</v>
       </c>
@@ -1902,7 +1914,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>78</v>
       </c>
@@ -1910,7 +1922,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>79</v>
       </c>
@@ -1918,7 +1930,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>80</v>
       </c>
@@ -1926,7 +1938,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>81</v>
       </c>
@@ -1934,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>82</v>
       </c>
@@ -1942,7 +1954,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>83</v>
       </c>
@@ -1950,7 +1962,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>84</v>
       </c>
@@ -1958,7 +1970,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>85</v>
       </c>
@@ -1966,7 +1978,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>86</v>
       </c>
@@ -1974,7 +1986,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>87</v>
       </c>
@@ -1982,7 +1994,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>305</v>
       </c>
@@ -1990,7 +2002,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>88</v>
       </c>
@@ -1998,7 +2010,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>89</v>
       </c>
@@ -2006,7 +2018,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>90</v>
       </c>
@@ -2014,7 +2026,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>91</v>
       </c>
@@ -2022,7 +2034,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>92</v>
       </c>
@@ -2030,7 +2042,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>93</v>
       </c>
@@ -2038,7 +2050,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>94</v>
       </c>
@@ -2046,7 +2058,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>95</v>
       </c>
@@ -2054,7 +2066,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>96</v>
       </c>
@@ -2062,7 +2074,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>97</v>
       </c>
@@ -2070,7 +2082,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>98</v>
       </c>
@@ -2078,7 +2090,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>99</v>
       </c>
@@ -2086,7 +2098,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>100</v>
       </c>
@@ -2094,7 +2106,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>306</v>
       </c>
@@ -2102,7 +2114,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>101</v>
       </c>
@@ -2110,7 +2122,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>102</v>
       </c>
@@ -2118,7 +2130,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>103</v>
       </c>
@@ -2126,7 +2138,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>104</v>
       </c>
@@ -2134,7 +2146,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>105</v>
       </c>
@@ -2142,7 +2154,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>106</v>
       </c>
@@ -2150,7 +2162,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>107</v>
       </c>
@@ -2158,7 +2170,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>108</v>
       </c>
@@ -2166,7 +2178,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>109</v>
       </c>
@@ -2174,7 +2186,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>110</v>
       </c>
@@ -2182,7 +2194,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>111</v>
       </c>
@@ -2190,7 +2202,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>112</v>
       </c>
@@ -2198,7 +2210,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>113</v>
       </c>
@@ -2206,7 +2218,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>114</v>
       </c>
@@ -2214,7 +2226,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>115</v>
       </c>
@@ -2222,7 +2234,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>116</v>
       </c>
@@ -2230,7 +2242,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>117</v>
       </c>
@@ -2238,7 +2250,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>118</v>
       </c>
@@ -2246,7 +2258,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>119</v>
       </c>
@@ -2254,7 +2266,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>120</v>
       </c>
@@ -2262,7 +2274,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>121</v>
       </c>
@@ -2270,7 +2282,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>122</v>
       </c>
@@ -2278,7 +2290,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>123</v>
       </c>
@@ -2286,7 +2298,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>124</v>
       </c>
@@ -2294,7 +2306,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>125</v>
       </c>
@@ -2302,7 +2314,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>126</v>
       </c>
@@ -2310,7 +2322,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>127</v>
       </c>
@@ -2318,7 +2330,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>128</v>
       </c>
@@ -2326,7 +2338,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>129</v>
       </c>
@@ -2334,7 +2346,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>130</v>
       </c>
@@ -2342,7 +2354,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>131</v>
       </c>
@@ -2350,7 +2362,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>132</v>
       </c>
@@ -2358,7 +2370,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>133</v>
       </c>
@@ -2366,7 +2378,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>134</v>
       </c>
@@ -2374,7 +2386,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>135</v>
       </c>
@@ -2382,7 +2394,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>136</v>
       </c>
@@ -2390,7 +2402,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>137</v>
       </c>
@@ -2398,7 +2410,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>138</v>
       </c>
@@ -2406,7 +2418,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>139</v>
       </c>
@@ -2414,7 +2426,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>140</v>
       </c>
@@ -2422,7 +2434,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>141</v>
       </c>
@@ -2430,7 +2442,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>142</v>
       </c>
@@ -2438,7 +2450,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>143</v>
       </c>
@@ -2446,7 +2458,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>144</v>
       </c>
@@ -2454,7 +2466,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>311</v>
       </c>
@@ -2462,7 +2474,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>145</v>
       </c>
@@ -2470,7 +2482,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>146</v>
       </c>
@@ -2478,7 +2490,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>147</v>
       </c>
@@ -2486,7 +2498,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>148</v>
       </c>
@@ -2494,7 +2506,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>149</v>
       </c>
@@ -2502,7 +2514,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>150</v>
       </c>
@@ -2510,7 +2522,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>151</v>
       </c>
@@ -2518,7 +2530,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>152</v>
       </c>
@@ -2526,7 +2538,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>153</v>
       </c>
@@ -2534,7 +2546,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>154</v>
       </c>
@@ -2542,7 +2554,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>155</v>
       </c>
@@ -2550,7 +2562,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>156</v>
       </c>
@@ -2558,7 +2570,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>157</v>
       </c>
@@ -2566,7 +2578,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>158</v>
       </c>
@@ -2574,7 +2586,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>159</v>
       </c>
@@ -2582,7 +2594,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>160</v>
       </c>
@@ -2590,7 +2602,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>161</v>
       </c>
@@ -2598,7 +2610,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>162</v>
       </c>
@@ -2606,7 +2618,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>163</v>
       </c>
@@ -2614,7 +2626,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>164</v>
       </c>
@@ -2622,7 +2634,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>165</v>
       </c>
@@ -2630,7 +2642,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>166</v>
       </c>
@@ -2638,7 +2650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>167</v>
       </c>
@@ -2646,7 +2658,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>168</v>
       </c>
@@ -2654,7 +2666,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>169</v>
       </c>
@@ -2662,7 +2674,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>170</v>
       </c>
@@ -2670,7 +2682,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>171</v>
       </c>
@@ -2678,7 +2690,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>172</v>
       </c>
@@ -2686,7 +2698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>173</v>
       </c>
@@ -2694,7 +2706,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>174</v>
       </c>
@@ -2702,7 +2714,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>175</v>
       </c>
@@ -2710,7 +2722,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>176</v>
       </c>
@@ -2718,7 +2730,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>177</v>
       </c>
@@ -2726,7 +2738,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>178</v>
       </c>
@@ -2734,7 +2746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>179</v>
       </c>
@@ -2742,7 +2754,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>180</v>
       </c>
@@ -2750,7 +2762,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>181</v>
       </c>
@@ -2758,7 +2770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>182</v>
       </c>
@@ -2766,7 +2778,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>183</v>
       </c>
@@ -2774,7 +2786,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>184</v>
       </c>
@@ -2782,7 +2794,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>185</v>
       </c>
@@ -2790,7 +2802,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>186</v>
       </c>
@@ -2798,7 +2810,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>187</v>
       </c>
@@ -2806,7 +2818,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>188</v>
       </c>
@@ -2814,7 +2826,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>189</v>
       </c>
@@ -2822,7 +2834,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>190</v>
       </c>
@@ -2830,7 +2842,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>191</v>
       </c>
@@ -2838,7 +2850,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>192</v>
       </c>
@@ -2846,7 +2858,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>193</v>
       </c>
@@ -2854,7 +2866,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>194</v>
       </c>
@@ -2862,7 +2874,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>195</v>
       </c>
@@ -2870,7 +2882,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>196</v>
       </c>
@@ -2878,7 +2890,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>197</v>
       </c>
@@ -2886,7 +2898,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>198</v>
       </c>
@@ -2894,7 +2906,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>199</v>
       </c>
@@ -2902,7 +2914,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>200</v>
       </c>
@@ -2910,7 +2922,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>201</v>
       </c>
@@ -2918,7 +2930,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>202</v>
       </c>
@@ -2926,7 +2938,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>203</v>
       </c>
@@ -2934,892 +2946,912 @@
         <v>15</v>
       </c>
     </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
+        <v>313</v>
+      </c>
+      <c r="B200" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
         <v>204</v>
       </c>
-      <c r="B200" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A201" t="s">
+      <c r="B201" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
         <v>205</v>
       </c>
-      <c r="B201" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A202" t="s">
+      <c r="B202" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
         <v>206</v>
       </c>
-      <c r="B202" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A203" t="s">
+      <c r="B203" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
         <v>207</v>
       </c>
-      <c r="B203" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A204" t="s">
+      <c r="B204" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
         <v>208</v>
       </c>
-      <c r="B204" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A205" t="s">
+      <c r="B205" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
         <v>209</v>
       </c>
-      <c r="B205" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A206" t="s">
+      <c r="B206" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
         <v>210</v>
       </c>
-      <c r="B206" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A207" t="s">
+      <c r="B207" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
         <v>211</v>
       </c>
-      <c r="B207" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A208" t="s">
+      <c r="B208" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
         <v>212</v>
       </c>
-      <c r="B208" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A209" t="s">
+      <c r="B209" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
         <v>213</v>
       </c>
-      <c r="B209" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A210" t="s">
+      <c r="B210" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
         <v>214</v>
       </c>
-      <c r="B210" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A211" t="s">
+      <c r="B211" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
         <v>215</v>
       </c>
-      <c r="B211" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A212" t="s">
+      <c r="B212" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
         <v>216</v>
       </c>
-      <c r="B212" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A213" t="s">
+      <c r="B213" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
         <v>217</v>
       </c>
-      <c r="B213" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A214" t="s">
+      <c r="B214" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
         <v>218</v>
       </c>
-      <c r="B214" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A215" t="s">
+      <c r="B215" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
         <v>219</v>
       </c>
-      <c r="B215" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A216" t="s">
+      <c r="B216" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
         <v>220</v>
       </c>
-      <c r="B216" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A217" t="s">
+      <c r="B217" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
         <v>221</v>
       </c>
-      <c r="B217" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A218" t="s">
+      <c r="B218" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
         <v>222</v>
       </c>
-      <c r="B218" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A219" t="s">
+      <c r="B219" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
         <v>223</v>
       </c>
-      <c r="B219" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A220" t="s">
+      <c r="B220" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
         <v>224</v>
       </c>
-      <c r="B220" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A221" t="s">
+      <c r="B221" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
         <v>225</v>
       </c>
-      <c r="B221" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A222" t="s">
+      <c r="B222" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A223" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B222" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A223" s="2" t="s">
+      <c r="B223" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
         <v>227</v>
       </c>
-      <c r="B223" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A224" t="s">
+      <c r="B224" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
         <v>228</v>
       </c>
-      <c r="B224" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A225" t="s">
+      <c r="B225" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
         <v>229</v>
       </c>
-      <c r="B225" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A226" t="s">
+      <c r="B226" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
         <v>230</v>
       </c>
-      <c r="B226" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A227" t="s">
+      <c r="B227" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
         <v>231</v>
       </c>
-      <c r="B227" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A228" t="s">
+      <c r="B228" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
         <v>232</v>
       </c>
-      <c r="B228" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A229" t="s">
+      <c r="B229" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
         <v>233</v>
       </c>
-      <c r="B229" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A230" t="s">
+      <c r="B230" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
         <v>234</v>
       </c>
-      <c r="B230" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A231" t="s">
+      <c r="B231" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
         <v>235</v>
       </c>
-      <c r="B231" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A232" t="s">
+      <c r="B232" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
         <v>236</v>
       </c>
-      <c r="B232" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A233" t="s">
+      <c r="B233" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
         <v>237</v>
       </c>
-      <c r="B233" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A234" t="s">
+      <c r="B234" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
         <v>238</v>
       </c>
-      <c r="B234" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A235" t="s">
+      <c r="B235" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
         <v>239</v>
       </c>
-      <c r="B235" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A236" t="s">
+      <c r="B236" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
         <v>20</v>
       </c>
-      <c r="B236" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A237" t="s">
+      <c r="B237" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
         <v>240</v>
       </c>
-      <c r="B237" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A238" t="s">
+      <c r="B238" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
         <v>241</v>
       </c>
-      <c r="B238" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A239" t="s">
+      <c r="B239" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
         <v>242</v>
       </c>
-      <c r="B239" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A240" t="s">
+      <c r="B240" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
         <v>243</v>
       </c>
-      <c r="B240" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A241" t="s">
+      <c r="B241" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
         <v>244</v>
       </c>
-      <c r="B241" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A242" t="s">
+      <c r="B242" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
         <v>245</v>
       </c>
-      <c r="B242" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A243" t="s">
+      <c r="B243" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
         <v>246</v>
       </c>
-      <c r="B243" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A244" t="s">
+      <c r="B244" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
         <v>247</v>
       </c>
-      <c r="B244" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A245" t="s">
+      <c r="B245" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
         <v>248</v>
       </c>
-      <c r="B245" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A246" t="s">
+      <c r="B246" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
         <v>249</v>
       </c>
-      <c r="B246" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A247" t="s">
+      <c r="B247" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
         <v>250</v>
       </c>
-      <c r="B247" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A248" t="s">
+      <c r="B248" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
         <v>251</v>
       </c>
-      <c r="B248" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A249" t="s">
+      <c r="B249" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
         <v>252</v>
       </c>
-      <c r="B249" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A250" t="s">
+      <c r="B250" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
         <v>253</v>
       </c>
-      <c r="B250" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A251" t="s">
+      <c r="B251" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
         <v>254</v>
       </c>
-      <c r="B251" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A252" t="s">
+      <c r="B252" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
         <v>255</v>
       </c>
-      <c r="B252" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A253" t="s">
+      <c r="B253" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
         <v>256</v>
       </c>
-      <c r="B253" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A254" t="s">
+      <c r="B254" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
         <v>257</v>
       </c>
-      <c r="B254" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A255" t="s">
+      <c r="B255" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
         <v>258</v>
       </c>
-      <c r="B255" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A256" t="s">
+      <c r="B256" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
         <v>259</v>
       </c>
-      <c r="B256" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A257" t="s">
+      <c r="B257" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A258" t="s">
         <v>260</v>
       </c>
-      <c r="B257" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A258" t="s">
+      <c r="B258" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
         <v>261</v>
       </c>
-      <c r="B258" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A259" t="s">
+      <c r="B259" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
         <v>262</v>
       </c>
-      <c r="B259" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A260" t="s">
+      <c r="B260" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
         <v>263</v>
       </c>
-      <c r="B260" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A261" t="s">
+      <c r="B261" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
         <v>264</v>
       </c>
-      <c r="B261" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A262" t="s">
+      <c r="B262" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
         <v>265</v>
       </c>
-      <c r="B262" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A263" t="s">
+      <c r="B263" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
         <v>266</v>
       </c>
-      <c r="B263" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A264" t="s">
+      <c r="B264" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A265" t="s">
         <v>267</v>
       </c>
-      <c r="B264" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A265" t="s">
+      <c r="B265" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
         <v>268</v>
       </c>
-      <c r="B265" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A266" t="s">
+      <c r="B266" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
         <v>269</v>
       </c>
-      <c r="B266" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A267" t="s">
+      <c r="B267" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
         <v>270</v>
       </c>
-      <c r="B267" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A268" t="s">
+      <c r="B268" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
         <v>271</v>
       </c>
-      <c r="B268" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A269" t="s">
+      <c r="B269" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
         <v>272</v>
       </c>
-      <c r="B269" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A270" t="s">
+      <c r="B270" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
         <v>273</v>
       </c>
-      <c r="B270" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A271" t="s">
+      <c r="B271" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
         <v>274</v>
       </c>
-      <c r="B271" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A272" t="s">
+      <c r="B272" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
         <v>275</v>
       </c>
-      <c r="B272" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A273" t="s">
+      <c r="B273" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
         <v>276</v>
       </c>
-      <c r="B273" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A274" t="s">
+      <c r="B274" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
         <v>277</v>
       </c>
-      <c r="B274" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A275" t="s">
+      <c r="B275" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
         <v>278</v>
       </c>
-      <c r="B275" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A276" t="s">
+      <c r="B276" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
         <v>279</v>
       </c>
-      <c r="B276" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A277" t="s">
+      <c r="B277" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
         <v>280</v>
       </c>
-      <c r="B277" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A278" t="s">
+      <c r="B278" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
         <v>281</v>
       </c>
-      <c r="B278" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A279" t="s">
+      <c r="B279" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
         <v>307</v>
       </c>
-      <c r="B279" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A280" t="s">
+      <c r="B280" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
         <v>282</v>
       </c>
-      <c r="B280" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A281" t="s">
+      <c r="B281" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
         <v>283</v>
       </c>
-      <c r="B281" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A282" t="s">
+      <c r="B282" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
         <v>284</v>
       </c>
-      <c r="B282" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A283" t="s">
+      <c r="B283" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
         <v>285</v>
       </c>
-      <c r="B283" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A284" t="s">
+      <c r="B284" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
         <v>286</v>
       </c>
-      <c r="B284" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A285" t="s">
+      <c r="B285" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>314</v>
+      </c>
+      <c r="B286" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
         <v>287</v>
       </c>
-      <c r="B285" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A286" t="s">
+      <c r="B287" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
         <v>288</v>
       </c>
-      <c r="B286" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A287" t="s">
+      <c r="B288" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>315</v>
+      </c>
+      <c r="B289" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
         <v>289</v>
       </c>
-      <c r="B287" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A288" t="s">
+      <c r="B290" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
         <v>290</v>
       </c>
-      <c r="B288" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A289" t="s">
+      <c r="B291" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
         <v>291</v>
       </c>
-      <c r="B289" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A290" t="s">
+      <c r="B292" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
         <v>292</v>
       </c>
-      <c r="B290" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A291" t="s">
+      <c r="B293" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A294" t="s">
         <v>293</v>
       </c>
-      <c r="B291" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A292" t="s">
+      <c r="B294" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
         <v>294</v>
       </c>
-      <c r="B292" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A293" t="s">
+      <c r="B295" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
         <v>312</v>
       </c>
-      <c r="B293" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A294" t="s">
+      <c r="B296" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
         <v>308</v>
       </c>
-      <c r="B294" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A295" t="s">
+      <c r="B297" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
         <v>295</v>
       </c>
-      <c r="B295" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A296" t="s">
+      <c r="B298" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
         <v>296</v>
       </c>
-      <c r="B296" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A297" t="s">
+      <c r="B299" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
         <v>297</v>
       </c>
-      <c r="B297" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A298" t="s">
+      <c r="B300" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
         <v>298</v>
       </c>
-      <c r="B298" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A299" t="s">
+      <c r="B301" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A302" t="s">
         <v>299</v>
       </c>
-      <c r="B299" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A300" t="s">
+      <c r="B302" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A303" t="s">
         <v>300</v>
       </c>
-      <c r="B300" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A301" t="s">
+      <c r="B303" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
         <v>301</v>
       </c>
-      <c r="B301" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A302" t="s">
+      <c r="B304" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
         <v>302</v>
       </c>
-      <c r="B302" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A303" t="s">
+      <c r="B305" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
         <v>309</v>
       </c>
-      <c r="B303" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A304" t="s">
+      <c r="B306" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
         <v>10</v>
       </c>
-      <c r="B304" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A305" t="s">
+      <c r="B307" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
         <v>303</v>
       </c>
-      <c r="B305" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A306" t="s">
+      <c r="B308" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A309" t="s">
         <v>304</v>
       </c>
-      <c r="B306" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A307" t="s">
+      <c r="B309" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A310" t="s">
         <v>4</v>
       </c>
-      <c r="B307" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A308" t="s">
+      <c r="B310" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A311" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A312" t="s">
         <v>5</v>
       </c>
-      <c r="B308" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A309" t="s">
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A313" t="s">
         <v>8</v>
       </c>
-      <c r="B309" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A310" t="s">
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A314" t="s">
         <v>26</v>
-      </c>
-      <c r="B310" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated care data (v71)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_care.xlsx
+++ b/src/data/routekaart_status_care.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{357B885A-BF94-45AB-9A3C-602A95A47A97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC6BA4B6-CBE8-4280-BBD1-A3592B1C88C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="17250" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="2590" yWindow="2270" windowWidth="35050" windowHeight="17670" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="317">
   <si>
     <t>Status inleveren routekaart</t>
   </si>
@@ -1348,13 +1348,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F40E7E-2647-4F3F-8219-3AF753B4033B}">
   <dimension ref="A1:B314"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="73.140625" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="1" max="1" width="73.1796875" customWidth="1"/>
+    <col min="2" max="2" width="31.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1362,7 +1362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1394,7 +1394,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1410,15 +1410,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -1442,7 +1442,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1474,15 +1474,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1498,15 +1498,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -1530,23 +1530,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>12</v>
       </c>
       <c r="B23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>36</v>
       </c>
       <c r="B24" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>6</v>
       </c>
@@ -1554,7 +1554,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>310</v>
       </c>
@@ -1562,7 +1562,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -1578,15 +1578,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>41</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -1618,15 +1618,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>44</v>
       </c>
       <c r="B34" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>46</v>
       </c>
@@ -1642,15 +1642,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>47</v>
       </c>
       <c r="B37" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>7</v>
       </c>
@@ -1666,15 +1666,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>13</v>
       </c>
@@ -1682,23 +1682,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>50</v>
       </c>
       <c r="B42" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>51</v>
       </c>
       <c r="B43" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -1722,23 +1722,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>55</v>
       </c>
       <c r="B47" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>56</v>
       </c>
       <c r="B48" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>25</v>
       </c>
@@ -1746,7 +1746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>57</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>58</v>
       </c>
@@ -1762,23 +1762,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>59</v>
       </c>
       <c r="B52" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>60</v>
       </c>
       <c r="B53" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -1786,15 +1786,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>62</v>
       </c>
       <c r="B55" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>63</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>64</v>
       </c>
@@ -1810,7 +1810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>65</v>
       </c>
@@ -1818,15 +1818,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>66</v>
       </c>
       <c r="B59" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>67</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>68</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>69</v>
       </c>
@@ -1850,23 +1850,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>70</v>
       </c>
       <c r="B63" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>71</v>
       </c>
       <c r="B64" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>72</v>
       </c>
@@ -1874,7 +1874,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>73</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>74</v>
       </c>
@@ -1890,7 +1890,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>75</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>76</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>77</v>
       </c>
@@ -1914,15 +1914,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>78</v>
       </c>
       <c r="B71" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>79</v>
       </c>
@@ -1930,7 +1930,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>80</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>81</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>82</v>
       </c>
@@ -1954,15 +1954,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>83</v>
       </c>
       <c r="B76" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>84</v>
       </c>
@@ -1970,7 +1970,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>85</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>86</v>
       </c>
@@ -1986,15 +1986,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>87</v>
       </c>
       <c r="B80" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>305</v>
       </c>
@@ -2002,7 +2002,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>88</v>
       </c>
@@ -2010,7 +2010,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>89</v>
       </c>
@@ -2018,23 +2018,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>90</v>
       </c>
       <c r="B84" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>91</v>
       </c>
       <c r="B85" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>92</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>93</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>94</v>
       </c>
@@ -2058,7 +2058,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>95</v>
       </c>
@@ -2066,15 +2066,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>96</v>
       </c>
       <c r="B90" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>97</v>
       </c>
@@ -2082,7 +2082,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>98</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>99</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>100</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>306</v>
       </c>
@@ -2114,7 +2114,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>101</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>102</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>103</v>
       </c>
@@ -2138,15 +2138,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>104</v>
       </c>
       <c r="B99" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>105</v>
       </c>
@@ -2154,23 +2154,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>106</v>
       </c>
       <c r="B101" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>107</v>
       </c>
       <c r="B102" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>108</v>
       </c>
@@ -2178,15 +2178,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>109</v>
       </c>
       <c r="B104" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>110</v>
       </c>
@@ -2194,23 +2194,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>111</v>
       </c>
       <c r="B106" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>112</v>
       </c>
       <c r="B107" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>113</v>
       </c>
@@ -2218,15 +2218,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>114</v>
       </c>
       <c r="B109" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>115</v>
       </c>
@@ -2234,23 +2234,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>116</v>
       </c>
       <c r="B111" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>117</v>
       </c>
       <c r="B112" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>118</v>
       </c>
@@ -2258,31 +2258,31 @@
         <v>15</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>119</v>
       </c>
       <c r="B114" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>120</v>
       </c>
       <c r="B115" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>121</v>
       </c>
       <c r="B116" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>122</v>
       </c>
@@ -2290,7 +2290,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>123</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>124</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>125</v>
       </c>
@@ -2314,7 +2314,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>126</v>
       </c>
@@ -2322,15 +2322,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>127</v>
       </c>
       <c r="B122" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>128</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>129</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>130</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>131</v>
       </c>
@@ -2362,7 +2362,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>132</v>
       </c>
@@ -2370,23 +2370,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>133</v>
       </c>
       <c r="B128" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>134</v>
       </c>
       <c r="B129" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>135</v>
       </c>
@@ -2394,23 +2394,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>136</v>
       </c>
       <c r="B131" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>137</v>
       </c>
       <c r="B132" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>138</v>
       </c>
@@ -2418,7 +2418,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>139</v>
       </c>
@@ -2426,7 +2426,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>140</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>141</v>
       </c>
@@ -2442,15 +2442,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>142</v>
       </c>
       <c r="B137" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>143</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>144</v>
       </c>
@@ -2466,7 +2466,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>311</v>
       </c>
@@ -2474,23 +2474,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>145</v>
       </c>
       <c r="B141" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>146</v>
       </c>
       <c r="B142" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>147</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>148</v>
       </c>
@@ -2506,31 +2506,31 @@
         <v>15</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>149</v>
       </c>
       <c r="B145" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>150</v>
       </c>
       <c r="B146" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>151</v>
       </c>
       <c r="B147" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>152</v>
       </c>
@@ -2538,7 +2538,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>153</v>
       </c>
@@ -2546,15 +2546,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>154</v>
       </c>
       <c r="B150" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>155</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>156</v>
       </c>
@@ -2570,15 +2570,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>157</v>
       </c>
       <c r="B153" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>158</v>
       </c>
@@ -2586,15 +2586,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>159</v>
       </c>
       <c r="B155" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>160</v>
       </c>
@@ -2602,7 +2602,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>161</v>
       </c>
@@ -2610,7 +2610,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>162</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>163</v>
       </c>
@@ -2626,23 +2626,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>164</v>
       </c>
       <c r="B160" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>165</v>
       </c>
       <c r="B161" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>166</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>167</v>
       </c>
@@ -2658,31 +2658,31 @@
         <v>16</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
         <v>168</v>
       </c>
       <c r="B164" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>169</v>
       </c>
       <c r="B165" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>170</v>
       </c>
       <c r="B166" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>171</v>
       </c>
@@ -2690,7 +2690,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>172</v>
       </c>
@@ -2698,15 +2698,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>173</v>
       </c>
       <c r="B169" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>174</v>
       </c>
@@ -2714,7 +2714,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>175</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>176</v>
       </c>
@@ -2730,7 +2730,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>177</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>178</v>
       </c>
@@ -2746,7 +2746,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>179</v>
       </c>
@@ -2754,7 +2754,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>180</v>
       </c>
@@ -2762,7 +2762,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>181</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>182</v>
       </c>
@@ -2778,31 +2778,31 @@
         <v>15</v>
       </c>
     </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>183</v>
       </c>
       <c r="B179" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>184</v>
       </c>
       <c r="B180" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>185</v>
       </c>
       <c r="B181" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>186</v>
       </c>
@@ -2810,7 +2810,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>187</v>
       </c>
@@ -2818,15 +2818,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>188</v>
       </c>
       <c r="B184" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>189</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>190</v>
       </c>
@@ -2842,7 +2842,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>191</v>
       </c>
@@ -2850,7 +2850,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>192</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>193</v>
       </c>
@@ -2866,7 +2866,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>194</v>
       </c>
@@ -2874,7 +2874,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>195</v>
       </c>
@@ -2882,7 +2882,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>196</v>
       </c>
@@ -2890,7 +2890,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>197</v>
       </c>
@@ -2898,7 +2898,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>198</v>
       </c>
@@ -2906,15 +2906,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>199</v>
       </c>
       <c r="B195" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>200</v>
       </c>
@@ -2922,15 +2922,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>201</v>
       </c>
       <c r="B197" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>202</v>
       </c>
@@ -2938,7 +2938,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
         <v>203</v>
       </c>
@@ -2946,7 +2946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
         <v>313</v>
       </c>
@@ -2954,15 +2954,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>204</v>
       </c>
       <c r="B201" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
         <v>205</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
         <v>206</v>
       </c>
@@ -2978,63 +2978,63 @@
         <v>15</v>
       </c>
     </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
         <v>207</v>
       </c>
       <c r="B204" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
         <v>208</v>
       </c>
       <c r="B205" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
         <v>209</v>
       </c>
       <c r="B206" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
         <v>210</v>
       </c>
       <c r="B207" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>211</v>
       </c>
       <c r="B208" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
         <v>212</v>
       </c>
       <c r="B209" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
         <v>213</v>
       </c>
       <c r="B210" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
         <v>214</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
         <v>215</v>
       </c>
@@ -3050,15 +3050,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
         <v>216</v>
       </c>
       <c r="B213" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
         <v>217</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
         <v>218</v>
       </c>
@@ -3074,31 +3074,31 @@
         <v>15</v>
       </c>
     </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
         <v>219</v>
       </c>
       <c r="B216" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>220</v>
       </c>
       <c r="B217" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>221</v>
       </c>
       <c r="B218" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>222</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>223</v>
       </c>
@@ -3114,23 +3114,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
         <v>224</v>
       </c>
       <c r="B221" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
         <v>225</v>
       </c>
       <c r="B222" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>226</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
         <v>227</v>
       </c>
@@ -3146,15 +3146,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
         <v>228</v>
       </c>
       <c r="B225" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
         <v>229</v>
       </c>
@@ -3162,47 +3162,47 @@
         <v>16</v>
       </c>
     </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
         <v>230</v>
       </c>
       <c r="B227" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
         <v>231</v>
       </c>
       <c r="B228" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
         <v>232</v>
       </c>
       <c r="B229" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
         <v>233</v>
       </c>
       <c r="B230" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
         <v>234</v>
       </c>
       <c r="B231" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
         <v>235</v>
       </c>
@@ -3210,31 +3210,31 @@
         <v>16</v>
       </c>
     </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
         <v>236</v>
       </c>
       <c r="B233" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
         <v>237</v>
       </c>
       <c r="B234" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
         <v>238</v>
       </c>
       <c r="B235" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
         <v>239</v>
       </c>
@@ -3242,15 +3242,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
         <v>20</v>
       </c>
       <c r="B237" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
         <v>240</v>
       </c>
@@ -3258,15 +3258,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
         <v>241</v>
       </c>
       <c r="B239" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
         <v>242</v>
       </c>
@@ -3274,15 +3274,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
         <v>243</v>
       </c>
       <c r="B241" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
         <v>244</v>
       </c>
@@ -3290,7 +3290,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
         <v>245</v>
       </c>
@@ -3298,23 +3298,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
         <v>246</v>
       </c>
       <c r="B244" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
         <v>247</v>
       </c>
       <c r="B245" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
         <v>248</v>
       </c>
@@ -3322,15 +3322,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
         <v>249</v>
       </c>
       <c r="B247" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
         <v>250</v>
       </c>
@@ -3338,23 +3338,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
         <v>251</v>
       </c>
       <c r="B249" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
         <v>252</v>
       </c>
       <c r="B250" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
         <v>253</v>
       </c>
@@ -3362,7 +3362,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
         <v>254</v>
       </c>
@@ -3370,7 +3370,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
         <v>255</v>
       </c>
@@ -3378,31 +3378,31 @@
         <v>15</v>
       </c>
     </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
         <v>256</v>
       </c>
       <c r="B254" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
         <v>257</v>
       </c>
       <c r="B255" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
         <v>258</v>
       </c>
       <c r="B256" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
         <v>259</v>
       </c>
@@ -3410,7 +3410,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
         <v>260</v>
       </c>
@@ -3418,15 +3418,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
         <v>261</v>
       </c>
       <c r="B259" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
         <v>262</v>
       </c>
@@ -3434,15 +3434,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
         <v>263</v>
       </c>
       <c r="B261" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
         <v>264</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
         <v>265</v>
       </c>
@@ -3458,7 +3458,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
         <v>266</v>
       </c>
@@ -3466,7 +3466,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
         <v>267</v>
       </c>
@@ -3474,7 +3474,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
         <v>268</v>
       </c>
@@ -3482,15 +3482,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
         <v>269</v>
       </c>
       <c r="B267" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
         <v>270</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
         <v>271</v>
       </c>
@@ -3506,31 +3506,31 @@
         <v>16</v>
       </c>
     </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
         <v>272</v>
       </c>
       <c r="B270" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
         <v>273</v>
       </c>
       <c r="B271" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
         <v>274</v>
       </c>
       <c r="B272" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
         <v>275</v>
       </c>
@@ -3538,71 +3538,71 @@
         <v>15</v>
       </c>
     </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
         <v>276</v>
       </c>
       <c r="B274" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
         <v>277</v>
       </c>
       <c r="B275" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
         <v>278</v>
       </c>
       <c r="B276" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
         <v>279</v>
       </c>
       <c r="B277" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
         <v>280</v>
       </c>
       <c r="B278" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
         <v>281</v>
       </c>
       <c r="B279" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
         <v>307</v>
       </c>
       <c r="B280" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
         <v>282</v>
       </c>
       <c r="B281" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
         <v>283</v>
       </c>
@@ -3610,15 +3610,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
         <v>284</v>
       </c>
       <c r="B283" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
         <v>285</v>
       </c>
@@ -3626,23 +3626,23 @@
         <v>16</v>
       </c>
     </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
         <v>286</v>
       </c>
       <c r="B285" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
         <v>314</v>
       </c>
       <c r="B286" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
         <v>287</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
         <v>288</v>
       </c>
@@ -3658,15 +3658,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
         <v>315</v>
       </c>
       <c r="B289" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
         <v>289</v>
       </c>
@@ -3674,7 +3674,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
         <v>290</v>
       </c>
@@ -3682,7 +3682,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
         <v>291</v>
       </c>
@@ -3690,7 +3690,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
         <v>292</v>
       </c>
@@ -3698,15 +3698,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
         <v>293</v>
       </c>
       <c r="B294" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
         <v>294</v>
       </c>
@@ -3714,7 +3714,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
         <v>312</v>
       </c>
@@ -3722,7 +3722,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
         <v>308</v>
       </c>
@@ -3730,23 +3730,23 @@
         <v>15</v>
       </c>
     </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
         <v>295</v>
       </c>
       <c r="B298" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
         <v>296</v>
       </c>
       <c r="B299" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
         <v>297</v>
       </c>
@@ -3754,15 +3754,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
         <v>298</v>
       </c>
       <c r="B301" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
         <v>299</v>
       </c>
@@ -3770,7 +3770,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
         <v>300</v>
       </c>
@@ -3778,15 +3778,15 @@
         <v>16</v>
       </c>
     </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
         <v>301</v>
       </c>
       <c r="B304" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
         <v>302</v>
       </c>
@@ -3794,15 +3794,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
         <v>309</v>
       </c>
       <c r="B306" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
         <v>10</v>
       </c>
@@ -3810,7 +3810,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
         <v>303</v>
       </c>
@@ -3818,7 +3818,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
         <v>304</v>
       </c>
@@ -3826,32 +3826,44 @@
         <v>16</v>
       </c>
     </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
         <v>4</v>
       </c>
       <c r="B310" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B311" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B312" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B313" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
         <v>26</v>
+      </c>
+      <c r="B314" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data correction: added Beacura
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_care.xlsx
+++ b/src/data/routekaart_status_care.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC6BA4B6-CBE8-4280-BBD1-A3592B1C88C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E2B2A47-00F5-4DA1-901A-D669BFDEB24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2590" yWindow="2270" windowWidth="35050" windowHeight="17670" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="5210" yWindow="430" windowWidth="27410" windowHeight="18630" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1919,7 +1919,7 @@
         <v>78</v>
       </c>
       <c r="B71" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Updated care data (v75)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_care.xlsx
+++ b/src/data/routekaart_status_care.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47796151-499F-4016-B2A2-03C3B77F5858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC2A338-F58B-45D5-B431-8B98B211CC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8390" yWindow="2990" windowWidth="27860" windowHeight="16420" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="5750" yWindow="4020" windowWidth="31690" windowHeight="15450" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="321">
   <si>
     <t>Status inleveren routekaart</t>
   </si>
@@ -986,6 +986,12 @@
   </si>
   <si>
     <t>Stichting Revant</t>
+  </si>
+  <si>
+    <t>Stichting Accare, Universitaire en Algemene Kinder- en Jeugdpsychiatrie Noord-Nederland</t>
+  </si>
+  <si>
+    <t>Zorgstichting 't Heem</t>
   </si>
 </sst>
 </file>
@@ -1353,7 +1359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F40E7E-2647-4F3F-8219-3AF753B4033B}">
-  <dimension ref="A1:B316"/>
+  <dimension ref="A1:B318"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="73.1796875" customWidth="1"/>
@@ -1613,7 +1619,7 @@
         <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
@@ -1722,31 +1728,31 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>53</v>
+        <v>319</v>
       </c>
       <c r="B46" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B47" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B48" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B49" t="s">
         <v>15</v>
@@ -1754,23 +1760,23 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="B50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="B51" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B52" t="s">
         <v>15</v>
@@ -1778,7 +1784,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B53" t="s">
         <v>15</v>
@@ -1786,7 +1792,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B54" t="s">
         <v>15</v>
@@ -1794,15 +1800,15 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B56" t="s">
         <v>16</v>
@@ -1810,7 +1816,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B57" t="s">
         <v>16</v>
@@ -1818,7 +1824,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B58" t="s">
         <v>16</v>
@@ -1826,15 +1832,15 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B59" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B60" t="s">
         <v>15</v>
@@ -1842,7 +1848,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B61" t="s">
         <v>15</v>
@@ -1850,7 +1856,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B62" t="s">
         <v>15</v>
@@ -1858,7 +1864,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B63" t="s">
         <v>15</v>
@@ -1866,7 +1872,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B64" t="s">
         <v>15</v>
@@ -1874,7 +1880,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B65" t="s">
         <v>15</v>
@@ -1882,23 +1888,23 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B66" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B67" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B68" t="s">
         <v>15</v>
@@ -1906,7 +1912,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B69" t="s">
         <v>15</v>
@@ -1914,7 +1920,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B70" t="s">
         <v>15</v>
@@ -1922,7 +1928,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B71" t="s">
         <v>15</v>
@@ -1930,7 +1936,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B72" t="s">
         <v>15</v>
@@ -1938,7 +1944,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B73" t="s">
         <v>15</v>
@@ -1946,7 +1952,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B74" t="s">
         <v>15</v>
@@ -1954,7 +1960,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B75" t="s">
         <v>15</v>
@@ -1962,7 +1968,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B76" t="s">
         <v>15</v>
@@ -1970,7 +1976,7 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B77" t="s">
         <v>15</v>
@@ -1978,7 +1984,7 @@
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B78" t="s">
         <v>15</v>
@@ -1986,7 +1992,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B79" t="s">
         <v>15</v>
@@ -1994,7 +2000,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B80" t="s">
         <v>15</v>
@@ -2002,15 +2008,15 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B81" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>305</v>
+        <v>87</v>
       </c>
       <c r="B82" t="s">
         <v>16</v>
@@ -2018,31 +2024,31 @@
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>88</v>
+        <v>305</v>
       </c>
       <c r="B83" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B84" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B85" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B86" t="s">
         <v>15</v>
@@ -2050,7 +2056,7 @@
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B87" t="s">
         <v>15</v>
@@ -2058,7 +2064,7 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B88" t="s">
         <v>15</v>
@@ -2066,7 +2072,7 @@
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B89" t="s">
         <v>15</v>
@@ -2074,15 +2080,15 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B90" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B91" t="s">
         <v>16</v>
@@ -2090,31 +2096,31 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B92" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B93" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B94" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B95" t="s">
         <v>15</v>
@@ -2122,7 +2128,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>306</v>
+        <v>100</v>
       </c>
       <c r="B96" t="s">
         <v>15</v>
@@ -2130,7 +2136,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>101</v>
+        <v>306</v>
       </c>
       <c r="B97" t="s">
         <v>15</v>
@@ -2138,7 +2144,7 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B98" t="s">
         <v>15</v>
@@ -2146,7 +2152,7 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B99" t="s">
         <v>15</v>
@@ -2154,7 +2160,7 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B100" t="s">
         <v>15</v>
@@ -2162,7 +2168,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B101" t="s">
         <v>15</v>
@@ -2170,63 +2176,63 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B102" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B103" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B104" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B105" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B106" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B107" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B108" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B109" t="s">
         <v>16</v>
@@ -2234,15 +2240,15 @@
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B110" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B111" t="s">
         <v>15</v>
@@ -2250,23 +2256,23 @@
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B112" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B113" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B114" t="s">
         <v>15</v>
@@ -2274,39 +2280,39 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B115" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B116" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B117" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B118" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B119" t="s">
         <v>15</v>
@@ -2314,7 +2320,7 @@
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B120" t="s">
         <v>15</v>
@@ -2322,7 +2328,7 @@
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B121" t="s">
         <v>15</v>
@@ -2330,7 +2336,7 @@
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B122" t="s">
         <v>15</v>
@@ -2338,7 +2344,7 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B123" t="s">
         <v>15</v>
@@ -2346,7 +2352,7 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B124" t="s">
         <v>15</v>
@@ -2354,7 +2360,7 @@
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B125" t="s">
         <v>15</v>
@@ -2362,7 +2368,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B126" t="s">
         <v>15</v>
@@ -2370,23 +2376,23 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B127" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B128" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B129" t="s">
         <v>15</v>
@@ -2394,7 +2400,7 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B130" t="s">
         <v>15</v>
@@ -2402,23 +2408,23 @@
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B131" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B132" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B133" t="s">
         <v>15</v>
@@ -2426,7 +2432,7 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B134" t="s">
         <v>15</v>
@@ -2434,7 +2440,7 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B135" t="s">
         <v>15</v>
@@ -2442,31 +2448,31 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B136" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B137" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B138" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B139" t="s">
         <v>16</v>
@@ -2474,7 +2480,7 @@
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B140" t="s">
         <v>16</v>
@@ -2482,7 +2488,7 @@
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>311</v>
+        <v>144</v>
       </c>
       <c r="B141" t="s">
         <v>16</v>
@@ -2490,23 +2496,23 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>145</v>
+        <v>311</v>
       </c>
       <c r="B142" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B144" t="s">
         <v>15</v>
@@ -2514,7 +2520,7 @@
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B145" t="s">
         <v>15</v>
@@ -2522,7 +2528,7 @@
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B146" t="s">
         <v>15</v>
@@ -2530,23 +2536,23 @@
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B149" t="s">
         <v>15</v>
@@ -2554,7 +2560,7 @@
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B150" t="s">
         <v>15</v>
@@ -2562,7 +2568,7 @@
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B151" t="s">
         <v>15</v>
@@ -2570,23 +2576,23 @@
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B154" t="s">
         <v>15</v>
@@ -2594,39 +2600,39 @@
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B159" t="s">
         <v>15</v>
@@ -2634,7 +2640,7 @@
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B160" t="s">
         <v>15</v>
@@ -2642,7 +2648,7 @@
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B161" t="s">
         <v>15</v>
@@ -2650,7 +2656,7 @@
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B162" t="s">
         <v>15</v>
@@ -2658,7 +2664,7 @@
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B163" t="s">
         <v>15</v>
@@ -2666,39 +2672,39 @@
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A164" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B168" t="s">
         <v>15</v>
@@ -2706,7 +2712,7 @@
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B169" t="s">
         <v>15</v>
@@ -2714,7 +2720,7 @@
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B170" t="s">
         <v>15</v>
@@ -2722,15 +2728,15 @@
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B172" t="s">
         <v>16</v>
@@ -2738,7 +2744,7 @@
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B173" t="s">
         <v>16</v>
@@ -2746,31 +2752,31 @@
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B177" t="s">
         <v>15</v>
@@ -2778,7 +2784,7 @@
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B178" t="s">
         <v>15</v>
@@ -2786,7 +2792,7 @@
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B179" t="s">
         <v>15</v>
@@ -2794,23 +2800,23 @@
     </row>
     <row r="180" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="181" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="182" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B182" t="s">
         <v>15</v>
@@ -2818,7 +2824,7 @@
     </row>
     <row r="183" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B183" t="s">
         <v>15</v>
@@ -2826,7 +2832,7 @@
     </row>
     <row r="184" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B184" t="s">
         <v>15</v>
@@ -2834,7 +2840,7 @@
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B185" t="s">
         <v>15</v>
@@ -2842,7 +2848,7 @@
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B186" t="s">
         <v>15</v>
@@ -2850,15 +2856,15 @@
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B188" t="s">
         <v>16</v>
@@ -2866,15 +2872,15 @@
     </row>
     <row r="189" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="190" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B190" t="s">
         <v>15</v>
@@ -2882,7 +2888,7 @@
     </row>
     <row r="191" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B191" t="s">
         <v>15</v>
@@ -2890,23 +2896,23 @@
     </row>
     <row r="192" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="193" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="194" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B194" t="s">
         <v>15</v>
@@ -2914,7 +2920,7 @@
     </row>
     <row r="195" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B195" t="s">
         <v>15</v>
@@ -2922,7 +2928,7 @@
     </row>
     <row r="196" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B196" t="s">
         <v>15</v>
@@ -2930,7 +2936,7 @@
     </row>
     <row r="197" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B197" t="s">
         <v>15</v>
@@ -2938,7 +2944,7 @@
     </row>
     <row r="198" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B198" t="s">
         <v>15</v>
@@ -2946,7 +2952,7 @@
     </row>
     <row r="199" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A199" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B199" t="s">
         <v>15</v>
@@ -2954,7 +2960,7 @@
     </row>
     <row r="200" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A200" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B200" t="s">
         <v>15</v>
@@ -2962,55 +2968,55 @@
     </row>
     <row r="201" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
-        <v>313</v>
+        <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="202" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A202" t="s">
-        <v>204</v>
+        <v>313</v>
       </c>
       <c r="B202" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="203" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A203" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B203" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="204" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A204" t="s">
-        <v>318</v>
+        <v>205</v>
       </c>
       <c r="B204" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="205" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A205" t="s">
-        <v>206</v>
+        <v>318</v>
       </c>
       <c r="B205" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="206" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A206" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B206" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B207" t="s">
         <v>15</v>
@@ -3018,7 +3024,7 @@
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B208" t="s">
         <v>15</v>
@@ -3026,7 +3032,7 @@
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B209" t="s">
         <v>15</v>
@@ -3034,31 +3040,31 @@
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B210" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B211" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B212" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B213" t="s">
         <v>15</v>
@@ -3066,15 +3072,15 @@
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B214" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B215" t="s">
         <v>16</v>
@@ -3082,15 +3088,15 @@
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B216" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B217" t="s">
         <v>15</v>
@@ -3098,7 +3104,7 @@
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B218" t="s">
         <v>15</v>
@@ -3106,23 +3112,23 @@
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B219" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B220" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B221" t="s">
         <v>15</v>
@@ -3130,7 +3136,7 @@
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B222" t="s">
         <v>15</v>
@@ -3138,7 +3144,7 @@
     </row>
     <row r="223" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B223" t="s">
         <v>15</v>
@@ -3146,7 +3152,7 @@
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B224" t="s">
         <v>15</v>
@@ -3154,15 +3160,15 @@
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B225" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B226" t="s">
         <v>16</v>
@@ -3170,15 +3176,15 @@
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B227" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B228" t="s">
         <v>15</v>
@@ -3186,23 +3192,23 @@
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B229" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B230" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B231" t="s">
         <v>15</v>
@@ -3210,31 +3216,31 @@
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B232" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B233" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B234" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B235" t="s">
         <v>16</v>
@@ -3242,31 +3248,31 @@
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B236" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B237" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B238" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
-        <v>20</v>
+        <v>239</v>
       </c>
       <c r="B239" t="s">
         <v>15</v>
@@ -3274,7 +3280,7 @@
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
-        <v>240</v>
+        <v>20</v>
       </c>
       <c r="B240" t="s">
         <v>15</v>
@@ -3282,7 +3288,7 @@
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B241" t="s">
         <v>15</v>
@@ -3290,15 +3296,15 @@
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B242" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B243" t="s">
         <v>16</v>
@@ -3306,15 +3312,15 @@
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B244" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B245" t="s">
         <v>15</v>
@@ -3322,7 +3328,7 @@
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B246" t="s">
         <v>15</v>
@@ -3330,23 +3336,23 @@
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B247" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B248" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B249" t="s">
         <v>15</v>
@@ -3354,15 +3360,15 @@
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B250" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B251" t="s">
         <v>16</v>
@@ -3370,15 +3376,15 @@
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B252" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B253" t="s">
         <v>15</v>
@@ -3386,7 +3392,7 @@
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B254" t="s">
         <v>15</v>
@@ -3394,7 +3400,7 @@
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B255" t="s">
         <v>15</v>
@@ -3402,7 +3408,7 @@
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B256" t="s">
         <v>15</v>
@@ -3410,7 +3416,7 @@
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B257" t="s">
         <v>15</v>
@@ -3418,23 +3424,23 @@
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B258" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B259" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B260" t="s">
         <v>15</v>
@@ -3442,7 +3448,7 @@
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B261" t="s">
         <v>15</v>
@@ -3450,7 +3456,7 @@
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B262" t="s">
         <v>15</v>
@@ -3458,7 +3464,7 @@
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B263" t="s">
         <v>15</v>
@@ -3466,23 +3472,23 @@
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B264" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B265" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B266" t="s">
         <v>15</v>
@@ -3490,7 +3496,7 @@
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B267" t="s">
         <v>15</v>
@@ -3498,7 +3504,7 @@
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B268" t="s">
         <v>15</v>
@@ -3506,7 +3512,7 @@
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B269" t="s">
         <v>15</v>
@@ -3514,7 +3520,7 @@
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B270" t="s">
         <v>15</v>
@@ -3522,15 +3528,15 @@
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B271" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B272" t="s">
         <v>16</v>
@@ -3538,31 +3544,31 @@
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B273" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B274" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B275" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B276" t="s">
         <v>15</v>
@@ -3570,31 +3576,31 @@
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B277" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B278" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B279" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B280" t="s">
         <v>16</v>
@@ -3602,15 +3608,15 @@
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B281" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>307</v>
+        <v>281</v>
       </c>
       <c r="B282" t="s">
         <v>15</v>
@@ -3618,7 +3624,7 @@
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>282</v>
+        <v>307</v>
       </c>
       <c r="B283" t="s">
         <v>15</v>
@@ -3626,7 +3632,7 @@
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B284" t="s">
         <v>15</v>
@@ -3634,31 +3640,31 @@
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B285" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B286" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B287" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>314</v>
+        <v>286</v>
       </c>
       <c r="B288" t="s">
         <v>16</v>
@@ -3666,23 +3672,23 @@
     </row>
     <row r="289" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
-        <v>287</v>
+        <v>314</v>
       </c>
       <c r="B289" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="290" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B290" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="291" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
-        <v>315</v>
+        <v>288</v>
       </c>
       <c r="B291" t="s">
         <v>16</v>
@@ -3690,47 +3696,47 @@
     </row>
     <row r="292" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
-        <v>289</v>
+        <v>315</v>
       </c>
       <c r="B292" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="293" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B293" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="294" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B294" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="295" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B295" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="296" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B296" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="297" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B297" t="s">
         <v>15</v>
@@ -3738,7 +3744,7 @@
     </row>
     <row r="298" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
-        <v>312</v>
+        <v>294</v>
       </c>
       <c r="B298" t="s">
         <v>15</v>
@@ -3746,7 +3752,7 @@
     </row>
     <row r="299" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="B299" t="s">
         <v>15</v>
@@ -3754,7 +3760,7 @@
     </row>
     <row r="300" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="B300" t="s">
         <v>15</v>
@@ -3762,7 +3768,7 @@
     </row>
     <row r="301" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B301" t="s">
         <v>15</v>
@@ -3770,7 +3776,7 @@
     </row>
     <row r="302" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B302" t="s">
         <v>15</v>
@@ -3778,39 +3784,39 @@
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B303" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="304" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B304" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="305" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B305" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="306" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B306" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="307" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B307" t="s">
         <v>15</v>
@@ -3818,23 +3824,23 @@
     </row>
     <row r="308" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="B308" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="309" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
-        <v>10</v>
+        <v>309</v>
       </c>
       <c r="B309" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="310" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
-        <v>303</v>
+        <v>10</v>
       </c>
       <c r="B310" t="s">
         <v>15</v>
@@ -3842,7 +3848,7 @@
     </row>
     <row r="311" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B311" t="s">
         <v>15</v>
@@ -3850,7 +3856,7 @@
     </row>
     <row r="312" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
-        <v>4</v>
+        <v>304</v>
       </c>
       <c r="B312" t="s">
         <v>15</v>
@@ -3858,7 +3864,7 @@
     </row>
     <row r="313" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="B313" t="s">
         <v>15</v>
@@ -3866,15 +3872,15 @@
     </row>
     <row r="314" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>5</v>
+        <v>316</v>
       </c>
       <c r="B314" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="315" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B315" t="s">
         <v>16</v>
@@ -3882,10 +3888,26 @@
     </row>
     <row r="316" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
+        <v>8</v>
+      </c>
+      <c r="B316" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A317" t="s">
         <v>26</v>
       </c>
-      <c r="B316" t="s">
-        <v>15</v>
+      <c r="B317" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A318" t="s">
+        <v>320</v>
+      </c>
+      <c r="B318" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated care data (v76)
</commit_message>
<xml_diff>
--- a/src/data/routekaart_status_care.xlsx
+++ b/src/data/routekaart_status_care.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC2A338-F58B-45D5-B431-8B98B211CC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E1283C-0038-47B1-B362-63E86CE87A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5750" yWindow="4020" windowWidth="31690" windowHeight="15450" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
+    <workbookView xWindow="8990" yWindow="3020" windowWidth="23770" windowHeight="15370" xr2:uid="{8CE8C91A-5D2B-429A-9150-16FF2E6CA716}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="326">
   <si>
     <t>Status inleveren routekaart</t>
   </si>
@@ -992,6 +992,21 @@
   </si>
   <si>
     <t>Zorgstichting 't Heem</t>
+  </si>
+  <si>
+    <t>Stichting RIBW Overijssel</t>
+  </si>
+  <si>
+    <t>Stichting TriviumMeulenbeltZorg</t>
+  </si>
+  <si>
+    <t>Stichting Vivantes Zorggroep</t>
+  </si>
+  <si>
+    <t>Stichting Zorgcollectief Zuidwest-Drenthe (ZZWD)</t>
+  </si>
+  <si>
+    <t>Zorgvilla's Duyvenstaete</t>
   </si>
 </sst>
 </file>
@@ -1359,7 +1374,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F40E7E-2647-4F3F-8219-3AF753B4033B}">
-  <dimension ref="A1:B318"/>
+  <dimension ref="A1:B323"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="73.1796875" customWidth="1"/>
@@ -1419,7 +1434,7 @@
         <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -1731,7 +1746,7 @@
         <v>319</v>
       </c>
       <c r="B46" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
@@ -3016,7 +3031,7 @@
     </row>
     <row r="207" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A207" t="s">
-        <v>207</v>
+        <v>321</v>
       </c>
       <c r="B207" t="s">
         <v>15</v>
@@ -3024,7 +3039,7 @@
     </row>
     <row r="208" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B208" t="s">
         <v>15</v>
@@ -3032,7 +3047,7 @@
     </row>
     <row r="209" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A209" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B209" t="s">
         <v>15</v>
@@ -3040,7 +3055,7 @@
     </row>
     <row r="210" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A210" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B210" t="s">
         <v>15</v>
@@ -3048,23 +3063,23 @@
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A211" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B211" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="212" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A212" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B212" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A213" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B213" t="s">
         <v>15</v>
@@ -3072,7 +3087,7 @@
     </row>
     <row r="214" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A214" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B214" t="s">
         <v>15</v>
@@ -3080,15 +3095,15 @@
     </row>
     <row r="215" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A215" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B215" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="216" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A216" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B216" t="s">
         <v>16</v>
@@ -3096,15 +3111,15 @@
     </row>
     <row r="217" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B217" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="218" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B218" t="s">
         <v>15</v>
@@ -3112,7 +3127,7 @@
     </row>
     <row r="219" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B219" t="s">
         <v>15</v>
@@ -3120,23 +3135,23 @@
     </row>
     <row r="220" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B220" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="221" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A221" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B221" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="222" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A222" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B222" t="s">
         <v>15</v>
@@ -3144,7 +3159,7 @@
     </row>
     <row r="223" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A223" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B223" t="s">
         <v>15</v>
@@ -3152,7 +3167,7 @@
     </row>
     <row r="224" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A224" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B224" t="s">
         <v>15</v>
@@ -3160,7 +3175,7 @@
     </row>
     <row r="225" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A225" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B225" t="s">
         <v>15</v>
@@ -3168,15 +3183,15 @@
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A226" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B226" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A227" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B227" t="s">
         <v>16</v>
@@ -3184,15 +3199,15 @@
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A228" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B228" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="229" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B229" t="s">
         <v>15</v>
@@ -3200,23 +3215,23 @@
     </row>
     <row r="230" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A230" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B230" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="231" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B231" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="232" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A232" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B232" t="s">
         <v>15</v>
@@ -3224,31 +3239,31 @@
     </row>
     <row r="233" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B233" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="234" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A234" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B234" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="235" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A235" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B235" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="236" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A236" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B236" t="s">
         <v>16</v>
@@ -3256,31 +3271,31 @@
     </row>
     <row r="237" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A237" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B237" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="238" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A238" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B238" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="239" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A239" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B239" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="240" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A240" t="s">
-        <v>20</v>
+        <v>239</v>
       </c>
       <c r="B240" t="s">
         <v>15</v>
@@ -3288,7 +3303,7 @@
     </row>
     <row r="241" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A241" t="s">
-        <v>240</v>
+        <v>20</v>
       </c>
       <c r="B241" t="s">
         <v>15</v>
@@ -3296,31 +3311,31 @@
     </row>
     <row r="242" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A242" t="s">
-        <v>241</v>
+        <v>322</v>
       </c>
       <c r="B242" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="243" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A243" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B243" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A244" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B244" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A245" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B245" t="s">
         <v>15</v>
@@ -3328,15 +3343,15 @@
     </row>
     <row r="246" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A246" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B246" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="247" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A247" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B247" t="s">
         <v>15</v>
@@ -3344,15 +3359,15 @@
     </row>
     <row r="248" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A248" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B248" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="249" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A249" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B249" t="s">
         <v>15</v>
@@ -3360,55 +3375,55 @@
     </row>
     <row r="250" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A250" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B250" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A251" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B251" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="252" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A252" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B252" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="253" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A253" t="s">
-        <v>252</v>
+        <v>323</v>
       </c>
       <c r="B253" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="254" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A254" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B254" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="255" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A255" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B255" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="256" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A256" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B256" t="s">
         <v>15</v>
@@ -3416,7 +3431,7 @@
     </row>
     <row r="257" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A257" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B257" t="s">
         <v>15</v>
@@ -3424,7 +3439,7 @@
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A258" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B258" t="s">
         <v>15</v>
@@ -3432,15 +3447,15 @@
     </row>
     <row r="259" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A259" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B259" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="260" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A260" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B260" t="s">
         <v>15</v>
@@ -3448,7 +3463,7 @@
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A261" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B261" t="s">
         <v>15</v>
@@ -3456,15 +3471,15 @@
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A262" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B262" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="263" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A263" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B263" t="s">
         <v>15</v>
@@ -3472,7 +3487,7 @@
     </row>
     <row r="264" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A264" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B264" t="s">
         <v>15</v>
@@ -3480,15 +3495,15 @@
     </row>
     <row r="265" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A265" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B265" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="266" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A266" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B266" t="s">
         <v>15</v>
@@ -3496,7 +3511,7 @@
     </row>
     <row r="267" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A267" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B267" t="s">
         <v>15</v>
@@ -3504,15 +3519,15 @@
     </row>
     <row r="268" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A268" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B268" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="269" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A269" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B269" t="s">
         <v>15</v>
@@ -3520,7 +3535,7 @@
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A270" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B270" t="s">
         <v>15</v>
@@ -3528,7 +3543,7 @@
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A271" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B271" t="s">
         <v>15</v>
@@ -3536,23 +3551,23 @@
     </row>
     <row r="272" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A272" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B272" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="273" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A273" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B273" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="274" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A274" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B274" t="s">
         <v>15</v>
@@ -3560,7 +3575,7 @@
     </row>
     <row r="275" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A275" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B275" t="s">
         <v>16</v>
@@ -3568,15 +3583,15 @@
     </row>
     <row r="276" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A276" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="B276" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A277" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B277" t="s">
         <v>15</v>
@@ -3584,7 +3599,7 @@
     </row>
     <row r="278" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A278" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B278" t="s">
         <v>16</v>
@@ -3592,7 +3607,7 @@
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A279" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B279" t="s">
         <v>15</v>
@@ -3600,15 +3615,15 @@
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A280" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="B280" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A281" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B281" t="s">
         <v>16</v>
@@ -3616,15 +3631,15 @@
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A282" t="s">
-        <v>281</v>
+        <v>324</v>
       </c>
       <c r="B282" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="283" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
-        <v>307</v>
+        <v>278</v>
       </c>
       <c r="B283" t="s">
         <v>15</v>
@@ -3632,31 +3647,31 @@
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B284" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B285" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B286" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
-        <v>285</v>
+        <v>307</v>
       </c>
       <c r="B287" t="s">
         <v>15</v>
@@ -3664,39 +3679,39 @@
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A288" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="B288" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="289" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A289" t="s">
-        <v>314</v>
+        <v>283</v>
       </c>
       <c r="B289" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="290" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A290" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B290" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="291" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A291" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B291" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="292" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A292" t="s">
-        <v>315</v>
+        <v>286</v>
       </c>
       <c r="B292" t="s">
         <v>16</v>
@@ -3704,31 +3719,31 @@
     </row>
     <row r="293" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A293" t="s">
-        <v>289</v>
+        <v>314</v>
       </c>
       <c r="B293" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="294" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A294" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B294" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="295" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A295" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B295" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="296" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A296" t="s">
-        <v>292</v>
+        <v>315</v>
       </c>
       <c r="B296" t="s">
         <v>16</v>
@@ -3736,7 +3751,7 @@
     </row>
     <row r="297" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A297" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B297" t="s">
         <v>15</v>
@@ -3744,15 +3759,15 @@
     </row>
     <row r="298" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A298" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B298" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="299" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A299" t="s">
-        <v>312</v>
+        <v>291</v>
       </c>
       <c r="B299" t="s">
         <v>15</v>
@@ -3760,15 +3775,15 @@
     </row>
     <row r="300" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A300" t="s">
-        <v>308</v>
+        <v>292</v>
       </c>
       <c r="B300" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="301" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A301" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B301" t="s">
         <v>15</v>
@@ -3776,7 +3791,7 @@
     </row>
     <row r="302" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A302" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B302" t="s">
         <v>15</v>
@@ -3784,7 +3799,7 @@
     </row>
     <row r="303" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A303" t="s">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="B303" t="s">
         <v>15</v>
@@ -3792,15 +3807,15 @@
     </row>
     <row r="304" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A304" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="B304" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="305" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A305" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B305" t="s">
         <v>15</v>
@@ -3808,15 +3823,15 @@
     </row>
     <row r="306" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A306" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="B306" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="307" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A307" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B307" t="s">
         <v>15</v>
@@ -3824,31 +3839,31 @@
     </row>
     <row r="308" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A308" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="B308" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="309" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A309" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="B309" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="310" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A310" t="s">
-        <v>10</v>
+        <v>300</v>
       </c>
       <c r="B310" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="311" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A311" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B311" t="s">
         <v>15</v>
@@ -3856,7 +3871,7 @@
     </row>
     <row r="312" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A312" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B312" t="s">
         <v>15</v>
@@ -3864,15 +3879,15 @@
     </row>
     <row r="313" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A313" t="s">
-        <v>4</v>
+        <v>309</v>
       </c>
       <c r="B313" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="314" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A314" t="s">
-        <v>316</v>
+        <v>10</v>
       </c>
       <c r="B314" t="s">
         <v>15</v>
@@ -3880,23 +3895,23 @@
     </row>
     <row r="315" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A315" t="s">
-        <v>5</v>
+        <v>303</v>
       </c>
       <c r="B315" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="316" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A316" t="s">
-        <v>8</v>
+        <v>304</v>
       </c>
       <c r="B316" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="317" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="B317" t="s">
         <v>15</v>
@@ -3904,10 +3919,50 @@
     </row>
     <row r="318" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A318" t="s">
+        <v>316</v>
+      </c>
+      <c r="B318" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A319" t="s">
+        <v>5</v>
+      </c>
+      <c r="B319" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A320" t="s">
+        <v>8</v>
+      </c>
+      <c r="B320" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A321" t="s">
+        <v>26</v>
+      </c>
+      <c r="B321" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A322" t="s">
         <v>320</v>
       </c>
-      <c r="B318" t="s">
-        <v>16</v>
+      <c r="B322" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A323" t="s">
+        <v>325</v>
+      </c>
+      <c r="B323" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>